<commit_message>
Update TeachingLoad workbook and add reference links.
Keep dataset and research links in sync for the garyprojects repository.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/dataset/TeachingLoad.xlsx
+++ b/dataset/TeachingLoad.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kwgar\aiTTO\dataset\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{78E19ACE-D03D-401C-87DD-A730CFC155A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FDFB0C7-3BEF-470E-A934-521E22B35D63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{B20823B3-F131-4B71-928E-DDCADA990BDD}"/>
   </bookViews>
@@ -187,6 +187,7 @@
     </xxl21:alternateUrls>
     <sheetNames>
       <sheetName val="Module arrangement - ABC Tech"/>
+      <sheetName val="Module arrangement - XYZ Tech"/>
       <sheetName val="Teaching Load"/>
       <sheetName val="Classroom"/>
       <sheetName val="Student sets"/>
@@ -314,9 +315,10 @@
           </cell>
         </row>
       </sheetData>
-      <sheetData sheetId="1"/>
-      <sheetData sheetId="2"/>
-      <sheetData sheetId="3"/>
+      <sheetData sheetId="1" refreshError="1"/>
+      <sheetData sheetId="2" refreshError="1"/>
+      <sheetData sheetId="3" refreshError="1"/>
+      <sheetData sheetId="4" refreshError="1"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>

</xml_diff>